<commit_message>
Actualizacion lun 04/05/2026 10:38:40,61
</commit_message>
<xml_diff>
--- a/mapping_propuesto.xlsx
+++ b/mapping_propuesto.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cd914253cd8ed602/EMPRESAS/Python Devs/finanzas-familia/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="296" documentId="11_D4AC3F2485E13763C1D08F2EA23E4392933AA06F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7AECD1C5-6427-40C6-93F9-F5614CE66D29}"/>
+  <xr:revisionPtr revIDLastSave="297" documentId="11_D4AC3F2485E13763C1D08F2EA23E4392933AA06F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DEEBA728-AE70-4D73-8C1E-8A792ADB9FC7}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1613,7 +1613,7 @@
       <c r="B16" s="7"/>
       <c r="C16" s="7"/>
       <c r="D16" s="8" t="s">
-        <v>17</v>
+        <v>52</v>
       </c>
       <c r="E16" s="9" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Actualizacion jue 07/05/2026  9:45:18,84
</commit_message>
<xml_diff>
--- a/mapping_propuesto.xlsx
+++ b/mapping_propuesto.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cd914253cd8ed602/EMPRESAS/Python Devs/finanzas-familia/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="297" documentId="11_D4AC3F2485E13763C1D08F2EA23E4392933AA06F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DEEBA728-AE70-4D73-8C1E-8A792ADB9FC7}"/>
+  <xr:revisionPtr revIDLastSave="298" documentId="11_D4AC3F2485E13763C1D08F2EA23E4392933AA06F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{11356409-6F81-4556-BEA6-D8FBCD599814}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instrucciones" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="226">
   <si>
     <t>Patrón texto</t>
   </si>
@@ -382,15 +382,6 @@
   </si>
   <si>
     <t>Bebé</t>
-  </si>
-  <si>
-    <t>Mapfre</t>
-  </si>
-  <si>
-    <t>Casa · Auto · Otro</t>
-  </si>
-  <si>
-    <t>Bonus</t>
   </si>
   <si>
     <t>Farmacia · Dentista · BCBS · Médico · Estudios · Otro</t>
@@ -1359,15 +1350,15 @@
         <v>77</v>
       </c>
       <c r="F2" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="B3" s="7"/>
       <c r="C3" s="7"/>
@@ -1378,15 +1369,15 @@
         <v>43</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="7"/>
@@ -1394,13 +1385,13 @@
         <v>36</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
@@ -1410,14 +1401,14 @@
       <c r="B5" s="7"/>
       <c r="C5" s="7"/>
       <c r="D5" s="8" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="E5" s="9"/>
       <c r="F5" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
@@ -1431,15 +1422,15 @@
       </c>
       <c r="E6" s="9"/>
       <c r="F6" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
@@ -1450,15 +1441,15 @@
         <v>62</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="B8" s="7"/>
       <c r="C8" s="7"/>
@@ -1469,15 +1460,15 @@
         <v>73</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
@@ -1488,10 +1479,10 @@
         <v>43</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G9" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
@@ -1505,15 +1496,15 @@
       </c>
       <c r="E10" s="9"/>
       <c r="F10" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="B11" s="7"/>
       <c r="C11" s="7"/>
@@ -1524,15 +1515,15 @@
         <v>72</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G11" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="B12" s="7"/>
       <c r="C12" s="7"/>
@@ -1540,13 +1531,13 @@
         <v>61</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G12" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
@@ -1562,10 +1553,10 @@
         <v>64</v>
       </c>
       <c r="F13" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G13" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
@@ -1581,10 +1572,10 @@
         <v>27</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G14" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
@@ -1597,13 +1588,13 @@
         <v>61</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
@@ -1619,15 +1610,15 @@
         <v>18</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G16" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="6" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
@@ -1635,13 +1626,13 @@
         <v>39</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G17" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
@@ -1654,13 +1645,13 @@
         <v>36</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G18" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
@@ -1673,13 +1664,13 @@
         <v>45</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G19" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
@@ -1695,10 +1686,10 @@
         <v>66</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
@@ -1712,29 +1703,29 @@
       </c>
       <c r="E21" s="9"/>
       <c r="F21" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G21" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="B22" s="7"/>
       <c r="C22" s="7"/>
       <c r="D22" s="8" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G22" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
@@ -1750,15 +1741,15 @@
         <v>80</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="B24" s="7"/>
       <c r="C24" s="7"/>
@@ -1767,10 +1758,10 @@
       </c>
       <c r="E24" s="9"/>
       <c r="F24" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G24" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
@@ -1784,16 +1775,16 @@
         <v>1500</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="F25" s="9" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="G25" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
@@ -1807,16 +1798,16 @@
         <v>5000</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="E26" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="F26" s="9" t="s">
         <v>177</v>
       </c>
-      <c r="F26" s="9" t="s">
-        <v>180</v>
-      </c>
       <c r="G26" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
@@ -1829,13 +1820,13 @@
         <v>36</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="F27" s="9" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="G27" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
@@ -1845,16 +1836,16 @@
       <c r="B28" s="7"/>
       <c r="C28" s="7"/>
       <c r="D28" s="8" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="G28" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
@@ -1864,16 +1855,16 @@
       <c r="B29" s="7"/>
       <c r="C29" s="7"/>
       <c r="D29" s="8" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="F29" s="9" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="G29" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
@@ -1883,21 +1874,21 @@
       <c r="B30" s="7"/>
       <c r="C30" s="7"/>
       <c r="D30" s="8" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="G30" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="6" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="B31" s="7"/>
       <c r="C31" s="7"/>
@@ -1905,32 +1896,32 @@
         <v>36</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="F31" s="9" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="G31" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="6" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B32" s="7"/>
       <c r="C32" s="7"/>
       <c r="D32" s="8" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="E32" s="9" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="G32" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
@@ -1940,16 +1931,16 @@
       <c r="B33" s="7"/>
       <c r="C33" s="7"/>
       <c r="D33" s="8" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="E33" s="9" t="s">
         <v>25</v>
       </c>
       <c r="F33" s="9" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="G33" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.3">
@@ -1965,15 +1956,15 @@
         <v>71</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G34" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="6" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="B35" s="7"/>
       <c r="C35" s="7"/>
@@ -1981,13 +1972,13 @@
         <v>41</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="F35" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G35" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
@@ -2003,15 +1994,15 @@
         <v>48</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G36" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" s="6" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="B37" s="7"/>
       <c r="C37" s="7"/>
@@ -2022,15 +2013,15 @@
         <v>27</v>
       </c>
       <c r="F37" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G37" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="6" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="B38" s="7"/>
       <c r="C38" s="7"/>
@@ -2038,13 +2029,13 @@
         <v>8</v>
       </c>
       <c r="E38" s="9" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G38" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.3">
@@ -2057,18 +2048,18 @@
         <v>8</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="F39" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G39" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="6" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="B40" s="7"/>
       <c r="C40" s="7"/>
@@ -2076,18 +2067,18 @@
         <v>52</v>
       </c>
       <c r="E40" s="9" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G40" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="6" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="B41" s="7"/>
       <c r="C41" s="7"/>
@@ -2095,18 +2086,18 @@
         <v>61</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="F41" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G41" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" s="6" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="B42" s="7"/>
       <c r="C42" s="7"/>
@@ -2117,10 +2108,10 @@
         <v>27</v>
       </c>
       <c r="F42" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G42" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.3">
@@ -2136,15 +2127,15 @@
         <v>27</v>
       </c>
       <c r="F43" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G43" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" s="6" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
@@ -2152,13 +2143,13 @@
         <v>36</v>
       </c>
       <c r="E44" s="9" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G44" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
@@ -2172,10 +2163,10 @@
       </c>
       <c r="E45" s="9"/>
       <c r="F45" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G45" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.3">
@@ -2191,10 +2182,10 @@
         <v>27</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G46" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.3">
@@ -2210,15 +2201,15 @@
         <v>31</v>
       </c>
       <c r="F47" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G47" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" s="6" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="B48" s="7"/>
       <c r="C48" s="7"/>
@@ -2229,10 +2220,10 @@
         <v>57</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G48" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
@@ -2248,29 +2239,29 @@
         <v>57</v>
       </c>
       <c r="F49" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G49" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" s="6" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B50" s="7"/>
       <c r="C50" s="7"/>
       <c r="D50" s="8" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="E50" s="9" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="F50" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G50" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.3">
@@ -2283,13 +2274,13 @@
         <v>11</v>
       </c>
       <c r="E51" s="9" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="F51" s="9" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="G51" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.3">
@@ -2302,32 +2293,32 @@
         <v>52</v>
       </c>
       <c r="E52" s="9" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="F52" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G52" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" s="6" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="B53" s="7"/>
       <c r="C53" s="7"/>
       <c r="D53" s="8" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="E53" s="9" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="F53" s="9" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="G53" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.3">
@@ -2343,10 +2334,10 @@
         <v>69</v>
       </c>
       <c r="F54" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G54" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.3">
@@ -2362,48 +2353,48 @@
         <v>27</v>
       </c>
       <c r="F55" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G55" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" s="6" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="B56" s="7"/>
       <c r="C56" s="7"/>
       <c r="D56" s="8" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="E56" s="9" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="F56" s="9" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="G56" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" s="6" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="B57" s="7"/>
       <c r="C57" s="7"/>
       <c r="D57" s="8" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="E57" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F57" s="9" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="G57" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.3">
@@ -2419,15 +2410,15 @@
         <v>75</v>
       </c>
       <c r="F58" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G58" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" s="6" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="B59" s="7"/>
       <c r="C59" s="7"/>
@@ -2435,13 +2426,13 @@
         <v>8</v>
       </c>
       <c r="E59" s="9" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="F59" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G59" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.3">
@@ -2454,18 +2445,18 @@
         <v>52</v>
       </c>
       <c r="E60" s="9" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="F60" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G60" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61" s="6" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B61" s="7"/>
       <c r="C61" s="7"/>
@@ -2473,13 +2464,13 @@
         <v>52</v>
       </c>
       <c r="E61" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F61" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G61" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -2498,13 +2489,13 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
         <x14:dataValidation type="list" allowBlank="1" errorTitle="Categoría inválida" error="Elegí una categoría de la lista de la hoja Categorías" xr:uid="{00000000-0002-0000-0100-000000000000}">
           <x14:formula1>
-            <xm:f>Categorías!$A$2:$A$28</xm:f>
+            <xm:f>Categorías!$A$2:$A$27</xm:f>
           </x14:formula1>
           <xm:sqref>D2:D686</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0100-000001000000}">
           <x14:formula1>
-            <xm:f>Categorías!$D$2:$D$63</xm:f>
+            <xm:f>Categorías!$D$2:$D$62</xm:f>
           </x14:formula1>
           <xm:sqref>E2:E686</xm:sqref>
         </x14:dataValidation>
@@ -2516,7 +2507,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D63"/>
+  <dimension ref="A1:D62"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -2603,117 +2594,117 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>119</v>
+        <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="D8" t="s">
-        <v>121</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>7</v>
+        <v>41</v>
       </c>
       <c r="B9" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="D9" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="B10" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D10" t="s">
-        <v>57</v>
+        <v>121</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="B11" t="s">
-        <v>123</v>
+        <v>114</v>
       </c>
       <c r="D11" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>8</v>
+        <v>52</v>
       </c>
       <c r="B12" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="D12" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>52</v>
+        <v>125</v>
       </c>
       <c r="B13" t="s">
         <v>126</v>
       </c>
       <c r="D13" t="s">
-        <v>127</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>128</v>
+        <v>17</v>
       </c>
       <c r="B14" t="s">
-        <v>129</v>
+        <v>18</v>
       </c>
       <c r="D14" t="s">
-        <v>14</v>
+        <v>127</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B15" t="s">
-        <v>18</v>
+        <v>128</v>
       </c>
       <c r="D15" t="s">
-        <v>130</v>
+        <v>55</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>21</v>
+        <v>129</v>
       </c>
       <c r="B16" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D16" t="s">
-        <v>55</v>
+        <v>27</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" t="s">
+        <v>131</v>
+      </c>
+      <c r="D17" t="s">
         <v>132</v>
-      </c>
-      <c r="B17" t="s">
-        <v>133</v>
-      </c>
-      <c r="D17" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>36</v>
+        <v>133</v>
       </c>
       <c r="B18" t="s">
         <v>134</v>
@@ -2724,54 +2715,54 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B19" t="s">
+        <v>114</v>
+      </c>
+      <c r="D19" t="s">
         <v>136</v>
-      </c>
-      <c r="B19" t="s">
-        <v>137</v>
-      </c>
-      <c r="D19" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>11</v>
+        <v>81</v>
       </c>
       <c r="B20" t="s">
         <v>114</v>
       </c>
       <c r="D20" t="s">
-        <v>139</v>
+        <v>42</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>81</v>
+        <v>137</v>
       </c>
       <c r="B21" t="s">
         <v>114</v>
       </c>
       <c r="D21" t="s">
-        <v>42</v>
+        <v>71</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B22" t="s">
         <v>114</v>
       </c>
       <c r="D22" t="s">
-        <v>71</v>
+        <v>139</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B23" t="s">
         <v>141</v>
-      </c>
-      <c r="B23" t="s">
-        <v>114</v>
       </c>
       <c r="D23" t="s">
         <v>142</v>
@@ -2782,229 +2773,218 @@
         <v>143</v>
       </c>
       <c r="B24" t="s">
+        <v>114</v>
+      </c>
+      <c r="D24" t="s">
         <v>144</v>
-      </c>
-      <c r="D24" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>146</v>
+        <v>40</v>
       </c>
       <c r="B25" t="s">
         <v>114</v>
       </c>
       <c r="D25" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>40</v>
+        <v>146</v>
       </c>
       <c r="B26" t="s">
         <v>114</v>
       </c>
       <c r="D26" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>149</v>
+        <v>171</v>
       </c>
       <c r="B27" t="s">
-        <v>114</v>
+        <v>170</v>
       </c>
       <c r="D27" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="B28" t="s">
-        <v>173</v>
-      </c>
       <c r="D28" t="s">
-        <v>151</v>
+        <v>43</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D29" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D30" t="s">
-        <v>37</v>
+        <v>80</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D31" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D32" t="s">
-        <v>75</v>
+        <v>149</v>
       </c>
     </row>
     <row r="33" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D33" t="s">
-        <v>152</v>
+        <v>24</v>
       </c>
     </row>
     <row r="34" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D34" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
     </row>
     <row r="35" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D35" t="s">
-        <v>15</v>
+        <v>150</v>
       </c>
     </row>
     <row r="36" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D36" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="37" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D37" t="s">
-        <v>154</v>
+        <v>77</v>
       </c>
     </row>
     <row r="38" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D38" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
     </row>
     <row r="39" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D39" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="40" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D40" t="s">
-        <v>62</v>
+        <v>152</v>
       </c>
     </row>
     <row r="41" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D41" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="42" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D42" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="43" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D43" t="s">
-        <v>157</v>
+        <v>50</v>
       </c>
     </row>
     <row r="44" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D44" t="s">
-        <v>50</v>
+        <v>78</v>
       </c>
     </row>
     <row r="45" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D45" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
     </row>
     <row r="46" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D46" t="s">
-        <v>66</v>
+        <v>155</v>
       </c>
     </row>
     <row r="47" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D47" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="48" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D48" t="s">
-        <v>159</v>
+        <v>31</v>
       </c>
     </row>
     <row r="49" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D49" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
     </row>
     <row r="50" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D50" t="s">
-        <v>18</v>
+        <v>47</v>
       </c>
     </row>
     <row r="51" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D51" t="s">
-        <v>47</v>
+        <v>157</v>
       </c>
     </row>
     <row r="52" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D52" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="53" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D53" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="54" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D54" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="55" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D55" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="56" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D56" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="57" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D57" t="s">
-        <v>165</v>
+        <v>59</v>
       </c>
     </row>
     <row r="58" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D58" t="s">
-        <v>59</v>
+        <v>163</v>
       </c>
     </row>
     <row r="59" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D59" t="s">
-        <v>166</v>
+        <v>72</v>
       </c>
     </row>
     <row r="60" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D60" t="s">
-        <v>72</v>
+        <v>51</v>
       </c>
     </row>
     <row r="61" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D61" t="s">
-        <v>51</v>
+        <v>164</v>
       </c>
     </row>
     <row r="62" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D62" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="63" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D63" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizacion mar 12/05/2026 11:20:32,26
</commit_message>
<xml_diff>
--- a/mapping_propuesto.xlsx
+++ b/mapping_propuesto.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cd914253cd8ed602/EMPRESAS/Python Devs/finanzas-familia/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="298" documentId="11_D4AC3F2485E13763C1D08F2EA23E4392933AA06F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{11356409-6F81-4556-BEA6-D8FBCD599814}"/>
+  <xr:revisionPtr revIDLastSave="306" documentId="11_D4AC3F2485E13763C1D08F2EA23E4392933AA06F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D3A0F224-6AF9-4C47-B7BF-0CEC041DCCD5}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instrucciones" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="228">
   <si>
     <t>Patrón texto</t>
   </si>
@@ -186,9 +186,6 @@
     <t>Social / Amigos</t>
   </si>
   <si>
-    <t>MISTERIO</t>
-  </si>
-  <si>
     <t>CAFE VD</t>
   </si>
   <si>
@@ -703,6 +700,15 @@
   </si>
   <si>
     <t>Dona Coxinha</t>
+  </si>
+  <si>
+    <t>Milanesas</t>
+  </si>
+  <si>
+    <t>Rudy</t>
+  </si>
+  <si>
+    <t>MISTERI</t>
   </si>
 </sst>
 </file>
@@ -769,7 +775,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -792,11 +798,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE5E7EB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE5E7EB"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -813,6 +830,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1127,7 +1145,7 @@
   <sheetData>
     <row r="1" spans="1:1" ht="17.399999999999999" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
@@ -1135,7 +1153,7 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
@@ -1143,17 +1161,17 @@
     </row>
     <row r="5" spans="1:1" ht="17.399999999999999" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
@@ -1161,7 +1179,7 @@
     </row>
     <row r="9" spans="1:1" ht="17.399999999999999" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
@@ -1169,17 +1187,17 @@
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.3">
@@ -1187,12 +1205,12 @@
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
@@ -1200,12 +1218,12 @@
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
@@ -1213,12 +1231,12 @@
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
@@ -1226,7 +1244,7 @@
     </row>
     <row r="24" spans="1:1" ht="17.399999999999999" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
@@ -1234,12 +1252,12 @@
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.3">
@@ -1247,22 +1265,22 @@
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
@@ -1270,12 +1288,12 @@
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.3">
@@ -1283,17 +1301,17 @@
     </row>
     <row r="37" spans="1:1" ht="17.399999999999999" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -1303,7 +1321,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:G62"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -1339,26 +1357,26 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B2" s="7"/>
       <c r="C2" s="7"/>
       <c r="D2" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F2" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B3" s="7"/>
       <c r="C3" s="7"/>
@@ -1369,15 +1387,15 @@
         <v>43</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="7"/>
@@ -1385,13 +1403,13 @@
         <v>36</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
@@ -1401,74 +1419,76 @@
       <c r="B5" s="7"/>
       <c r="C5" s="7"/>
       <c r="D5" s="8" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E5" s="9"/>
       <c r="F5" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="G5" s="9" t="s">
         <v>180</v>
-      </c>
-      <c r="G5" s="9" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B6" s="7"/>
       <c r="C6" s="7"/>
       <c r="D6" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="E6" s="9"/>
+      <c r="E6" s="9" t="s">
+        <v>226</v>
+      </c>
       <c r="F6" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
       <c r="D7" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="E7" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="E7" s="9" t="s">
-        <v>62</v>
-      </c>
       <c r="F7" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B8" s="7"/>
       <c r="C8" s="7"/>
       <c r="D8" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
@@ -1479,10 +1499,10 @@
         <v>43</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G9" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
@@ -1496,67 +1516,67 @@
       </c>
       <c r="E10" s="9"/>
       <c r="F10" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B11" s="7"/>
       <c r="C11" s="7"/>
       <c r="D11" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G11" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B12" s="7"/>
       <c r="C12" s="7"/>
       <c r="D12" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G12" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B13" s="7"/>
       <c r="C13" s="7"/>
       <c r="D13" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F13" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G13" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
@@ -1572,29 +1592,29 @@
         <v>27</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G14" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B15" s="7"/>
       <c r="C15" s="7"/>
       <c r="D15" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
@@ -1610,15 +1630,15 @@
         <v>18</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G16" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
@@ -1626,13 +1646,13 @@
         <v>39</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G17" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
@@ -1645,13 +1665,13 @@
         <v>36</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G18" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
@@ -1664,37 +1684,37 @@
         <v>45</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G19" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
       <c r="D20" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B21" s="7"/>
       <c r="C21" s="7"/>
@@ -1703,53 +1723,53 @@
       </c>
       <c r="E21" s="9"/>
       <c r="F21" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G21" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B22" s="7"/>
       <c r="C22" s="7"/>
       <c r="D22" s="8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G22" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B23" s="7"/>
       <c r="C23" s="7"/>
       <c r="D23" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B24" s="7"/>
       <c r="C24" s="7"/>
@@ -1758,10 +1778,10 @@
       </c>
       <c r="E24" s="9"/>
       <c r="F24" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G24" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
@@ -1775,16 +1795,16 @@
         <v>1500</v>
       </c>
       <c r="D25" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="E25" s="9" t="s">
         <v>172</v>
       </c>
-      <c r="E25" s="9" t="s">
-        <v>173</v>
-      </c>
       <c r="F25" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G25" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
@@ -1798,16 +1818,16 @@
         <v>5000</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G26" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
@@ -1820,13 +1840,13 @@
         <v>36</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F27" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G27" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
@@ -1836,16 +1856,16 @@
       <c r="B28" s="7"/>
       <c r="C28" s="7"/>
       <c r="D28" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G28" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
@@ -1855,16 +1875,16 @@
       <c r="B29" s="7"/>
       <c r="C29" s="7"/>
       <c r="D29" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F29" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G29" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
@@ -1874,21 +1894,21 @@
       <c r="B30" s="7"/>
       <c r="C30" s="7"/>
       <c r="D30" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E30" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="F30" s="9" t="s">
         <v>176</v>
       </c>
-      <c r="F30" s="9" t="s">
-        <v>177</v>
-      </c>
       <c r="G30" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B31" s="7"/>
       <c r="C31" s="7"/>
@@ -1896,32 +1916,32 @@
         <v>36</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F31" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G31" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="6" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B32" s="7"/>
       <c r="C32" s="7"/>
       <c r="D32" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E32" s="9" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G32" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
@@ -1931,40 +1951,40 @@
       <c r="B33" s="7"/>
       <c r="C33" s="7"/>
       <c r="D33" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E33" s="9" t="s">
         <v>25</v>
       </c>
       <c r="F33" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G33" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B34" s="7"/>
       <c r="C34" s="7"/>
       <c r="D34" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E34" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G34" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="6" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B35" s="7"/>
       <c r="C35" s="7"/>
@@ -1972,13 +1992,13 @@
         <v>41</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F35" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G35" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
@@ -1994,15 +2014,15 @@
         <v>48</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G36" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B37" s="7"/>
       <c r="C37" s="7"/>
@@ -2013,15 +2033,15 @@
         <v>27</v>
       </c>
       <c r="F37" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G37" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="6" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B38" s="7"/>
       <c r="C38" s="7"/>
@@ -2029,13 +2049,13 @@
         <v>8</v>
       </c>
       <c r="E38" s="9" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G38" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.3">
@@ -2048,18 +2068,18 @@
         <v>8</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="F39" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G39" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="6" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B40" s="7"/>
       <c r="C40" s="7"/>
@@ -2067,37 +2087,37 @@
         <v>52</v>
       </c>
       <c r="E40" s="9" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G40" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="6" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B41" s="7"/>
       <c r="C41" s="7"/>
       <c r="D41" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F41" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G41" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" s="6" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B42" s="7"/>
       <c r="C42" s="7"/>
@@ -2108,10 +2128,10 @@
         <v>27</v>
       </c>
       <c r="F42" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G42" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.3">
@@ -2127,15 +2147,15 @@
         <v>27</v>
       </c>
       <c r="F43" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G43" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" s="6" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
@@ -2143,13 +2163,13 @@
         <v>36</v>
       </c>
       <c r="E44" s="9" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G44" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
@@ -2163,10 +2183,10 @@
       </c>
       <c r="E45" s="9"/>
       <c r="F45" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G45" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.3">
@@ -2182,10 +2202,10 @@
         <v>27</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G46" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.3">
@@ -2201,15 +2221,15 @@
         <v>31</v>
       </c>
       <c r="F47" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G47" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" s="6" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B48" s="7"/>
       <c r="C48" s="7"/>
@@ -2217,18 +2237,18 @@
         <v>52</v>
       </c>
       <c r="E48" s="9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G48" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B49" s="7"/>
       <c r="C49" s="7"/>
@@ -2236,32 +2256,32 @@
         <v>52</v>
       </c>
       <c r="E49" s="9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F49" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G49" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B50" s="7"/>
       <c r="C50" s="7"/>
       <c r="D50" s="8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E50" s="9" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F50" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G50" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.3">
@@ -2274,18 +2294,18 @@
         <v>11</v>
       </c>
       <c r="E51" s="9" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F51" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G51" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" s="6" t="s">
-        <v>53</v>
+        <v>227</v>
       </c>
       <c r="B52" s="7"/>
       <c r="C52" s="7"/>
@@ -2293,51 +2313,51 @@
         <v>52</v>
       </c>
       <c r="E52" s="9" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F52" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G52" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" s="6" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B53" s="7"/>
       <c r="C53" s="7"/>
       <c r="D53" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E53" s="9" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F53" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G53" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" s="6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B54" s="7"/>
       <c r="C54" s="7"/>
       <c r="D54" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E54" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F54" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G54" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.3">
@@ -2353,72 +2373,72 @@
         <v>27</v>
       </c>
       <c r="F55" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G55" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" s="6" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B56" s="7"/>
       <c r="C56" s="7"/>
       <c r="D56" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E56" s="9" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F56" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G56" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" s="6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B57" s="7"/>
       <c r="C57" s="7"/>
       <c r="D57" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E57" s="9" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F57" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G57" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B58" s="7"/>
       <c r="C58" s="7"/>
       <c r="D58" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E58" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F58" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G58" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" s="6" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B59" s="7"/>
       <c r="C59" s="7"/>
@@ -2426,18 +2446,18 @@
         <v>8</v>
       </c>
       <c r="E59" s="9" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="F59" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G59" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B60" s="7"/>
       <c r="C60" s="7"/>
@@ -2445,18 +2465,18 @@
         <v>52</v>
       </c>
       <c r="E60" s="9" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="F60" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G60" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61" s="6" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B61" s="7"/>
       <c r="C61" s="7"/>
@@ -2464,13 +2484,30 @@
         <v>52</v>
       </c>
       <c r="E61" s="9" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="F61" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G61" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A62">
+        <v>3481838</v>
+      </c>
+      <c r="D62" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="E62" s="12" t="s">
+        <v>225</v>
+      </c>
+      <c r="F62" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="G62" s="12" t="s">
+        <v>177</v>
       </c>
     </row>
   </sheetData>
@@ -2520,18 +2557,18 @@
         <v>3</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="D1" s="10" t="s">
         <v>109</v>
-      </c>
-      <c r="D1" s="10" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D2" t="s">
         <v>48</v>
@@ -2542,10 +2579,10 @@
         <v>45</v>
       </c>
       <c r="B3" t="s">
+        <v>111</v>
+      </c>
+      <c r="D3" t="s">
         <v>112</v>
-      </c>
-      <c r="D3" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -2553,10 +2590,10 @@
         <v>35</v>
       </c>
       <c r="B4" t="s">
+        <v>113</v>
+      </c>
+      <c r="D4" t="s">
         <v>114</v>
-      </c>
-      <c r="D4" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -2564,21 +2601,21 @@
         <v>39</v>
       </c>
       <c r="B5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B6" t="s">
+        <v>113</v>
+      </c>
+      <c r="D6" t="s">
         <v>117</v>
-      </c>
-      <c r="B6" t="s">
-        <v>114</v>
-      </c>
-      <c r="D6" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
@@ -2586,10 +2623,10 @@
         <v>44</v>
       </c>
       <c r="B7" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -2597,7 +2634,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D8" t="s">
         <v>49</v>
@@ -2608,10 +2645,10 @@
         <v>41</v>
       </c>
       <c r="B9" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -2619,10 +2656,10 @@
         <v>26</v>
       </c>
       <c r="B10" t="s">
+        <v>119</v>
+      </c>
+      <c r="D10" t="s">
         <v>120</v>
-      </c>
-      <c r="D10" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -2630,10 +2667,10 @@
         <v>8</v>
       </c>
       <c r="B11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D11" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
@@ -2641,18 +2678,18 @@
         <v>52</v>
       </c>
       <c r="B12" t="s">
+        <v>122</v>
+      </c>
+      <c r="D12" t="s">
         <v>123</v>
-      </c>
-      <c r="D12" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B13" t="s">
         <v>125</v>
-      </c>
-      <c r="B13" t="s">
-        <v>126</v>
       </c>
       <c r="D13" t="s">
         <v>14</v>
@@ -2666,7 +2703,7 @@
         <v>18</v>
       </c>
       <c r="D14" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
@@ -2674,18 +2711,18 @@
         <v>21</v>
       </c>
       <c r="B15" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D15" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B16" t="s">
         <v>129</v>
-      </c>
-      <c r="B16" t="s">
-        <v>130</v>
       </c>
       <c r="D16" t="s">
         <v>27</v>
@@ -2696,21 +2733,21 @@
         <v>36</v>
       </c>
       <c r="B17" t="s">
+        <v>130</v>
+      </c>
+      <c r="D17" t="s">
         <v>131</v>
-      </c>
-      <c r="D17" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B18" t="s">
         <v>133</v>
       </c>
-      <c r="B18" t="s">
+      <c r="D18" t="s">
         <v>134</v>
-      </c>
-      <c r="D18" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
@@ -2718,18 +2755,18 @@
         <v>11</v>
       </c>
       <c r="B19" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D19" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B20" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D20" t="s">
         <v>42</v>
@@ -2737,46 +2774,46 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B21" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D21" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B22" t="s">
+        <v>113</v>
+      </c>
+      <c r="D22" t="s">
         <v>138</v>
-      </c>
-      <c r="B22" t="s">
-        <v>114</v>
-      </c>
-      <c r="D22" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B23" t="s">
         <v>140</v>
       </c>
-      <c r="B23" t="s">
+      <c r="D23" t="s">
         <v>141</v>
-      </c>
-      <c r="D23" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B24" t="s">
+        <v>113</v>
+      </c>
+      <c r="D24" t="s">
         <v>143</v>
-      </c>
-      <c r="B24" t="s">
-        <v>114</v>
-      </c>
-      <c r="D24" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
@@ -2784,32 +2821,32 @@
         <v>40</v>
       </c>
       <c r="B25" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D25" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B26" t="s">
+        <v>113</v>
+      </c>
+      <c r="D26" t="s">
         <v>146</v>
-      </c>
-      <c r="B26" t="s">
-        <v>114</v>
-      </c>
-      <c r="D26" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B27" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D27" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
@@ -2824,17 +2861,17 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D30" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D31" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D32" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="33" spans="4:4" x14ac:dyDescent="0.3">
@@ -2849,42 +2886,42 @@
     </row>
     <row r="35" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D35" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="36" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D36" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="37" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D37" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="38" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D38" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="39" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D39" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="40" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D40" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="41" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D41" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="42" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D42" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="43" spans="4:4" x14ac:dyDescent="0.3">
@@ -2894,22 +2931,22 @@
     </row>
     <row r="44" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D44" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="45" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D45" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="46" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D46" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="47" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D47" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="48" spans="4:4" x14ac:dyDescent="0.3">
@@ -2929,47 +2966,47 @@
     </row>
     <row r="51" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D51" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="52" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D52" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="53" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D53" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="54" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D54" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="55" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D55" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="56" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D56" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="57" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D57" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="58" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D58" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="59" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D59" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="60" spans="4:4" x14ac:dyDescent="0.3">
@@ -2979,12 +3016,12 @@
     </row>
     <row r="61" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D61" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="62" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D62" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizacion mié 20/05/2026 14:25:55,67
</commit_message>
<xml_diff>
--- a/mapping_propuesto.xlsx
+++ b/mapping_propuesto.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cd914253cd8ed602/EMPRESAS/Python Devs/finanzas-familia/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="306" documentId="11_D4AC3F2485E13763C1D08F2EA23E4392933AA06F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D3A0F224-6AF9-4C47-B7BF-0CEC041DCCD5}"/>
+  <xr:revisionPtr revIDLastSave="308" documentId="11_D4AC3F2485E13763C1D08F2EA23E4392933AA06F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{13B123BA-98BF-4A09-8C35-0A85DC818885}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="229">
   <si>
     <t>Patrón texto</t>
   </si>
@@ -709,6 +709,9 @@
   </si>
   <si>
     <t>MISTERI</t>
+  </si>
+  <si>
+    <t>TIENDA INLGE</t>
   </si>
 </sst>
 </file>
@@ -813,7 +816,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -830,7 +833,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1321,7 +1327,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G62"/>
+  <dimension ref="A1:G63"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -2508,6 +2514,17 @@
       </c>
       <c r="G62" s="12" t="s">
         <v>177</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A63" s="13" t="s">
+        <v>228</v>
+      </c>
+      <c r="D63" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="E63" s="9" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizacion lun 01/06/2026 15:15:52,07
</commit_message>
<xml_diff>
--- a/mapping_propuesto.xlsx
+++ b/mapping_propuesto.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cd914253cd8ed602/EMPRESAS/Python Devs/finanzas-familia/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="308" documentId="11_D4AC3F2485E13763C1D08F2EA23E4392933AA06F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{13B123BA-98BF-4A09-8C35-0A85DC818885}"/>
+  <xr:revisionPtr revIDLastSave="333" documentId="11_D4AC3F2485E13763C1D08F2EA23E4392933AA06F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{932CB609-2C98-4018-835A-1FD9E36CBEE6}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,12 +20,25 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Reglas!$A$1:$G$61</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="235">
   <si>
     <t>Patrón texto</t>
   </si>
@@ -712,6 +725,24 @@
   </si>
   <si>
     <t>TIENDA INLGE</t>
+  </si>
+  <si>
+    <t>CAMBIOST</t>
+  </si>
+  <si>
+    <t>Jardinero</t>
+  </si>
+  <si>
+    <t>MOVIE</t>
+  </si>
+  <si>
+    <t>RIOGAS</t>
+  </si>
+  <si>
+    <t>Garrafa</t>
+  </si>
+  <si>
+    <t>Uruing</t>
   </si>
 </sst>
 </file>
@@ -816,7 +847,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -834,9 +865,13 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1327,7 +1362,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G63"/>
+  <dimension ref="A1:G67"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -2525,6 +2560,84 @@
       </c>
       <c r="E63" s="9" t="s">
         <v>71</v>
+      </c>
+      <c r="F63" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="G63" s="12" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A64" s="13" t="s">
+        <v>229</v>
+      </c>
+      <c r="B64">
+        <v>1200</v>
+      </c>
+      <c r="C64">
+        <v>1200</v>
+      </c>
+      <c r="D64" t="s">
+        <v>230</v>
+      </c>
+      <c r="E64" s="12"/>
+      <c r="F64" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="G64" s="12" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A65" s="14" t="s">
+        <v>231</v>
+      </c>
+      <c r="D65" t="s">
+        <v>52</v>
+      </c>
+      <c r="E65" t="s">
+        <v>54</v>
+      </c>
+      <c r="F65" s="15" t="s">
+        <v>179</v>
+      </c>
+      <c r="G65" s="15" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A66" s="14" t="s">
+        <v>232</v>
+      </c>
+      <c r="D66" t="s">
+        <v>36</v>
+      </c>
+      <c r="E66" t="s">
+        <v>233</v>
+      </c>
+      <c r="F66" s="15" t="s">
+        <v>179</v>
+      </c>
+      <c r="G66" s="15" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A67">
+        <v>1935968</v>
+      </c>
+      <c r="D67" t="s">
+        <v>80</v>
+      </c>
+      <c r="E67" t="s">
+        <v>234</v>
+      </c>
+      <c r="F67" s="15" t="s">
+        <v>179</v>
+      </c>
+      <c r="G67" s="15" t="s">
+        <v>180</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizacion lun 01/06/2026 21:31:16,27
</commit_message>
<xml_diff>
--- a/mapping_propuesto.xlsx
+++ b/mapping_propuesto.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cd914253cd8ed602/EMPRESAS/Python Devs/finanzas-familia/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="333" documentId="11_D4AC3F2485E13763C1D08F2EA23E4392933AA06F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{932CB609-2C98-4018-835A-1FD9E36CBEE6}"/>
+  <xr:revisionPtr revIDLastSave="370" documentId="11_D4AC3F2485E13763C1D08F2EA23E4392933AA06F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9D4D0259-A2C9-4B09-BB33-A9F76F706174}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
     <sheet name="Categorías" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Reglas!$A$1:$G$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Reglas!$A$1:$G$60</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="236">
   <si>
     <t>Patrón texto</t>
   </si>
@@ -583,9 +583,6 @@
     <t>Ingresos</t>
   </si>
   <si>
-    <t>DEB. VARIOS VISA-ILINK</t>
-  </si>
-  <si>
     <t>S.E.M.M.</t>
   </si>
   <si>
@@ -743,6 +740,12 @@
   </si>
   <si>
     <t>Uruing</t>
+  </si>
+  <si>
+    <t>C.J.P.P</t>
+  </si>
+  <si>
+    <t>SEGURO DE VIDA</t>
   </si>
 </sst>
 </file>
@@ -847,7 +850,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -868,10 +871,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1362,7 +1361,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G67"/>
+  <dimension ref="A1:G70"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -1417,7 +1416,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B3" s="7"/>
       <c r="C3" s="7"/>
@@ -1480,7 +1479,7 @@
         <v>52</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F6" s="9" t="s">
         <v>179</v>
@@ -1491,7 +1490,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
@@ -1510,7 +1509,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B8" s="7"/>
       <c r="C8" s="7"/>
@@ -1529,7 +1528,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
@@ -1565,7 +1564,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B11" s="7"/>
       <c r="C11" s="7"/>
@@ -1584,7 +1583,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B12" s="7"/>
       <c r="C12" s="7"/>
@@ -1592,7 +1591,7 @@
         <v>60</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F12" s="9" t="s">
         <v>179</v>
@@ -1649,7 +1648,7 @@
         <v>60</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>179</v>
@@ -1679,7 +1678,7 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
@@ -1687,7 +1686,7 @@
         <v>39</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F17" s="9" t="s">
         <v>179</v>
@@ -1706,7 +1705,7 @@
         <v>36</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>179</v>
@@ -1725,7 +1724,7 @@
         <v>45</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F19" s="9" t="s">
         <v>179</v>
@@ -1772,7 +1771,7 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B22" s="7"/>
       <c r="C22" s="7"/>
@@ -1780,7 +1779,7 @@
         <v>132</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F22" s="9" t="s">
         <v>179</v>
@@ -1809,17 +1808,23 @@
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>181</v>
-      </c>
-      <c r="B24" s="7"/>
-      <c r="C24" s="7"/>
-      <c r="D24" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="E24" s="9"/>
+      <c r="A24" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B24" s="7">
+        <v>800</v>
+      </c>
+      <c r="C24" s="7">
+        <v>1500</v>
+      </c>
+      <c r="D24" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="E24" s="9" t="s">
+        <v>172</v>
+      </c>
       <c r="F24" s="9" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="G24" s="9" t="s">
         <v>177</v>
@@ -1830,16 +1835,16 @@
         <v>16</v>
       </c>
       <c r="B25" s="7">
-        <v>800</v>
+        <v>4000</v>
       </c>
       <c r="C25" s="7">
-        <v>1500</v>
+        <v>5000</v>
       </c>
       <c r="D25" s="11" t="s">
         <v>171</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F25" s="9" t="s">
         <v>176</v>
@@ -1850,19 +1855,15 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B26" s="7">
-        <v>4000</v>
-      </c>
-      <c r="C26" s="7">
-        <v>5000</v>
-      </c>
-      <c r="D26" s="11" t="s">
-        <v>171</v>
+        <v>12</v>
+      </c>
+      <c r="B26" s="7"/>
+      <c r="C26" s="7"/>
+      <c r="D26" s="8" t="s">
+        <v>36</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>173</v>
+        <v>196</v>
       </c>
       <c r="F26" s="9" t="s">
         <v>176</v>
@@ -1873,15 +1874,15 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="6" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="B27" s="7"/>
       <c r="C27" s="7"/>
       <c r="D27" s="8" t="s">
-        <v>36</v>
+        <v>170</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>176</v>
@@ -1892,7 +1893,7 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="6" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B28" s="7"/>
       <c r="C28" s="7"/>
@@ -1900,7 +1901,7 @@
         <v>170</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>199</v>
+        <v>178</v>
       </c>
       <c r="F28" s="9" t="s">
         <v>176</v>
@@ -1911,7 +1912,7 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B29" s="7"/>
       <c r="C29" s="7"/>
@@ -1919,7 +1920,7 @@
         <v>170</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="F29" s="9" t="s">
         <v>176</v>
@@ -1930,15 +1931,15 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="6" t="s">
-        <v>22</v>
+        <v>197</v>
       </c>
       <c r="B30" s="7"/>
       <c r="C30" s="7"/>
       <c r="D30" s="8" t="s">
-        <v>170</v>
+        <v>36</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="F30" s="9" t="s">
         <v>176</v>
@@ -1949,15 +1950,15 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="6" t="s">
-        <v>198</v>
+        <v>174</v>
       </c>
       <c r="B31" s="7"/>
       <c r="C31" s="7"/>
       <c r="D31" s="8" t="s">
-        <v>36</v>
+        <v>170</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>176</v>
@@ -1968,7 +1969,7 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="6" t="s">
-        <v>174</v>
+        <v>25</v>
       </c>
       <c r="B32" s="7"/>
       <c r="C32" s="7"/>
@@ -1976,7 +1977,7 @@
         <v>170</v>
       </c>
       <c r="E32" s="9" t="s">
-        <v>174</v>
+        <v>25</v>
       </c>
       <c r="F32" s="9" t="s">
         <v>176</v>
@@ -1987,18 +1988,18 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="6" t="s">
-        <v>25</v>
+        <v>69</v>
       </c>
       <c r="B33" s="7"/>
       <c r="C33" s="7"/>
       <c r="D33" s="8" t="s">
-        <v>170</v>
+        <v>60</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>25</v>
+        <v>70</v>
       </c>
       <c r="F33" s="9" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="G33" s="9" t="s">
         <v>177</v>
@@ -2006,18 +2007,18 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="6" t="s">
-        <v>69</v>
+        <v>181</v>
       </c>
       <c r="B34" s="7"/>
       <c r="C34" s="7"/>
       <c r="D34" s="8" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="E34" s="9" t="s">
-        <v>70</v>
+        <v>199</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="G34" s="9" t="s">
         <v>177</v>
@@ -2025,18 +2026,18 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="6" t="s">
-        <v>182</v>
+        <v>48</v>
       </c>
       <c r="B35" s="7"/>
       <c r="C35" s="7"/>
       <c r="D35" s="8" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>200</v>
+        <v>48</v>
       </c>
       <c r="F35" s="9" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="G35" s="9" t="s">
         <v>177</v>
@@ -2044,15 +2045,15 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="6" t="s">
-        <v>48</v>
+        <v>200</v>
       </c>
       <c r="B36" s="7"/>
       <c r="C36" s="7"/>
       <c r="D36" s="8" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="E36" s="9" t="s">
-        <v>48</v>
+        <v>27</v>
       </c>
       <c r="F36" s="9" t="s">
         <v>179</v>
@@ -2068,10 +2069,10 @@
       <c r="B37" s="7"/>
       <c r="C37" s="7"/>
       <c r="D37" s="8" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>27</v>
+        <v>223</v>
       </c>
       <c r="F37" s="9" t="s">
         <v>179</v>
@@ -2082,7 +2083,7 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="6" t="s">
-        <v>202</v>
+        <v>9</v>
       </c>
       <c r="B38" s="7"/>
       <c r="C38" s="7"/>
@@ -2090,7 +2091,7 @@
         <v>8</v>
       </c>
       <c r="E38" s="9" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="F38" s="9" t="s">
         <v>179</v>
@@ -2101,15 +2102,15 @@
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" s="6" t="s">
-        <v>9</v>
+        <v>202</v>
       </c>
       <c r="B39" s="7"/>
       <c r="C39" s="7"/>
       <c r="D39" s="8" t="s">
-        <v>8</v>
+        <v>52</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>223</v>
+        <v>203</v>
       </c>
       <c r="F39" s="9" t="s">
         <v>179</v>
@@ -2120,15 +2121,15 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B40" s="7"/>
       <c r="C40" s="7"/>
       <c r="D40" s="8" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="E40" s="9" t="s">
-        <v>204</v>
+        <v>138</v>
       </c>
       <c r="F40" s="9" t="s">
         <v>179</v>
@@ -2144,10 +2145,10 @@
       <c r="B41" s="7"/>
       <c r="C41" s="7"/>
       <c r="D41" s="8" t="s">
-        <v>60</v>
+        <v>26</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>138</v>
+        <v>27</v>
       </c>
       <c r="F41" s="9" t="s">
         <v>179</v>
@@ -2158,7 +2159,7 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" s="6" t="s">
-        <v>206</v>
+        <v>28</v>
       </c>
       <c r="B42" s="7"/>
       <c r="C42" s="7"/>
@@ -2177,15 +2178,15 @@
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" s="6" t="s">
-        <v>28</v>
+        <v>206</v>
       </c>
       <c r="B43" s="7"/>
       <c r="C43" s="7"/>
       <c r="D43" s="8" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="E43" s="9" t="s">
-        <v>27</v>
+        <v>207</v>
       </c>
       <c r="F43" s="9" t="s">
         <v>179</v>
@@ -2196,16 +2197,14 @@
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" s="6" t="s">
-        <v>207</v>
+        <v>34</v>
       </c>
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
       <c r="D44" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="E44" s="9" t="s">
-        <v>208</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="E44" s="9"/>
       <c r="F44" s="9" t="s">
         <v>179</v>
       </c>
@@ -2215,14 +2214,16 @@
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="6" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B45" s="7"/>
       <c r="C45" s="7"/>
       <c r="D45" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="E45" s="9"/>
+        <v>26</v>
+      </c>
+      <c r="E45" s="9" t="s">
+        <v>27</v>
+      </c>
       <c r="F45" s="9" t="s">
         <v>179</v>
       </c>
@@ -2232,18 +2233,18 @@
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B46" s="7"/>
       <c r="C46" s="7"/>
       <c r="D46" s="8" t="s">
-        <v>26</v>
+        <v>52</v>
       </c>
       <c r="E46" s="9" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="G46" s="9" t="s">
         <v>177</v>
@@ -2251,7 +2252,7 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" s="6" t="s">
-        <v>30</v>
+        <v>208</v>
       </c>
       <c r="B47" s="7"/>
       <c r="C47" s="7"/>
@@ -2259,7 +2260,7 @@
         <v>52</v>
       </c>
       <c r="E47" s="9" t="s">
-        <v>31</v>
+        <v>56</v>
       </c>
       <c r="F47" s="9" t="s">
         <v>179</v>
@@ -2270,7 +2271,7 @@
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" s="6" t="s">
-        <v>209</v>
+        <v>59</v>
       </c>
       <c r="B48" s="7"/>
       <c r="C48" s="7"/>
@@ -2289,15 +2290,15 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" s="6" t="s">
-        <v>59</v>
+        <v>209</v>
       </c>
       <c r="B49" s="7"/>
       <c r="C49" s="7"/>
       <c r="D49" s="8" t="s">
-        <v>52</v>
+        <v>132</v>
       </c>
       <c r="E49" s="9" t="s">
-        <v>56</v>
+        <v>210</v>
       </c>
       <c r="F49" s="9" t="s">
         <v>179</v>
@@ -2308,18 +2309,18 @@
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" s="6" t="s">
-        <v>210</v>
+        <v>13</v>
       </c>
       <c r="B50" s="7"/>
       <c r="C50" s="7"/>
       <c r="D50" s="8" t="s">
-        <v>132</v>
+        <v>11</v>
       </c>
       <c r="E50" s="9" t="s">
         <v>211</v>
       </c>
       <c r="F50" s="9" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="G50" s="9" t="s">
         <v>177</v>
@@ -2327,18 +2328,18 @@
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" s="6" t="s">
-        <v>13</v>
+        <v>226</v>
       </c>
       <c r="B51" s="7"/>
       <c r="C51" s="7"/>
       <c r="D51" s="8" t="s">
-        <v>11</v>
+        <v>52</v>
       </c>
       <c r="E51" s="9" t="s">
         <v>212</v>
       </c>
       <c r="F51" s="9" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="G51" s="9" t="s">
         <v>177</v>
@@ -2346,18 +2347,18 @@
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" s="6" t="s">
-        <v>227</v>
+        <v>213</v>
       </c>
       <c r="B52" s="7"/>
       <c r="C52" s="7"/>
       <c r="D52" s="8" t="s">
-        <v>52</v>
+        <v>170</v>
       </c>
       <c r="E52" s="9" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F52" s="9" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="G52" s="9" t="s">
         <v>177</v>
@@ -2365,18 +2366,18 @@
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" s="6" t="s">
-        <v>214</v>
+        <v>67</v>
       </c>
       <c r="B53" s="7"/>
       <c r="C53" s="7"/>
       <c r="D53" s="8" t="s">
-        <v>170</v>
+        <v>60</v>
       </c>
       <c r="E53" s="9" t="s">
-        <v>215</v>
+        <v>68</v>
       </c>
       <c r="F53" s="9" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="G53" s="9" t="s">
         <v>177</v>
@@ -2384,15 +2385,15 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" s="6" t="s">
-        <v>67</v>
+        <v>32</v>
       </c>
       <c r="B54" s="7"/>
       <c r="C54" s="7"/>
       <c r="D54" s="8" t="s">
-        <v>60</v>
+        <v>26</v>
       </c>
       <c r="E54" s="9" t="s">
-        <v>68</v>
+        <v>27</v>
       </c>
       <c r="F54" s="9" t="s">
         <v>179</v>
@@ -2403,18 +2404,18 @@
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" s="6" t="s">
-        <v>32</v>
+        <v>215</v>
       </c>
       <c r="B55" s="7"/>
       <c r="C55" s="7"/>
       <c r="D55" s="8" t="s">
-        <v>26</v>
+        <v>170</v>
       </c>
       <c r="E55" s="9" t="s">
-        <v>27</v>
+        <v>216</v>
       </c>
       <c r="F55" s="9" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="G55" s="9" t="s">
         <v>177</v>
@@ -2422,7 +2423,7 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" s="6" t="s">
-        <v>216</v>
+        <v>168</v>
       </c>
       <c r="B56" s="7"/>
       <c r="C56" s="7"/>
@@ -2430,7 +2431,7 @@
         <v>170</v>
       </c>
       <c r="E56" s="9" t="s">
-        <v>217</v>
+        <v>169</v>
       </c>
       <c r="F56" s="9" t="s">
         <v>176</v>
@@ -2441,18 +2442,18 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" s="6" t="s">
-        <v>168</v>
+        <v>73</v>
       </c>
       <c r="B57" s="7"/>
       <c r="C57" s="7"/>
       <c r="D57" s="8" t="s">
-        <v>170</v>
+        <v>60</v>
       </c>
       <c r="E57" s="9" t="s">
-        <v>169</v>
+        <v>74</v>
       </c>
       <c r="F57" s="9" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="G57" s="9" t="s">
         <v>177</v>
@@ -2460,15 +2461,15 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58" s="6" t="s">
-        <v>73</v>
+        <v>217</v>
       </c>
       <c r="B58" s="7"/>
       <c r="C58" s="7"/>
       <c r="D58" s="8" t="s">
-        <v>60</v>
+        <v>8</v>
       </c>
       <c r="E58" s="9" t="s">
-        <v>74</v>
+        <v>218</v>
       </c>
       <c r="F58" s="9" t="s">
         <v>179</v>
@@ -2479,12 +2480,12 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" s="6" t="s">
-        <v>218</v>
+        <v>55</v>
       </c>
       <c r="B59" s="7"/>
       <c r="C59" s="7"/>
       <c r="D59" s="8" t="s">
-        <v>8</v>
+        <v>52</v>
       </c>
       <c r="E59" s="9" t="s">
         <v>219</v>
@@ -2498,7 +2499,7 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60" s="6" t="s">
-        <v>55</v>
+        <v>220</v>
       </c>
       <c r="B60" s="7"/>
       <c r="C60" s="7"/>
@@ -2506,7 +2507,7 @@
         <v>52</v>
       </c>
       <c r="E60" s="9" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="F60" s="9" t="s">
         <v>179</v>
@@ -2516,33 +2517,31 @@
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A61" s="6" t="s">
-        <v>221</v>
-      </c>
-      <c r="B61" s="7"/>
-      <c r="C61" s="7"/>
+      <c r="A61">
+        <v>3481838</v>
+      </c>
       <c r="D61" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="E61" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="F61" s="9" t="s">
-        <v>179</v>
-      </c>
-      <c r="G61" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="E61" s="12" t="s">
+        <v>224</v>
+      </c>
+      <c r="F61" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="G61" s="12" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A62">
-        <v>3481838</v>
+      <c r="A62" s="13" t="s">
+        <v>227</v>
       </c>
       <c r="D62" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="E62" s="12" t="s">
-        <v>225</v>
+      <c r="E62" s="9" t="s">
+        <v>71</v>
       </c>
       <c r="F62" s="12" t="s">
         <v>179</v>
@@ -2555,12 +2554,16 @@
       <c r="A63" s="13" t="s">
         <v>228</v>
       </c>
-      <c r="D63" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="E63" s="9" t="s">
-        <v>71</v>
-      </c>
+      <c r="B63">
+        <v>1200</v>
+      </c>
+      <c r="C63">
+        <v>1200</v>
+      </c>
+      <c r="D63" t="s">
+        <v>229</v>
+      </c>
+      <c r="E63" s="12"/>
       <c r="F63" s="12" t="s">
         <v>179</v>
       </c>
@@ -2570,18 +2573,14 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A64" s="13" t="s">
-        <v>229</v>
-      </c>
-      <c r="B64">
-        <v>1200</v>
-      </c>
-      <c r="C64">
-        <v>1200</v>
+        <v>230</v>
       </c>
       <c r="D64" t="s">
-        <v>230</v>
-      </c>
-      <c r="E64" s="12"/>
+        <v>52</v>
+      </c>
+      <c r="E64" t="s">
+        <v>54</v>
+      </c>
       <c r="F64" s="12" t="s">
         <v>179</v>
       </c>
@@ -2590,63 +2589,108 @@
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A65" s="14" t="s">
+      <c r="A65" s="13" t="s">
         <v>231</v>
       </c>
       <c r="D65" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="E65" t="s">
-        <v>54</v>
-      </c>
-      <c r="F65" s="15" t="s">
-        <v>179</v>
-      </c>
-      <c r="G65" s="15" t="s">
+        <v>232</v>
+      </c>
+      <c r="F65" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="G65" s="12" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A66" s="14" t="s">
-        <v>232</v>
+      <c r="A66">
+        <v>1935968</v>
       </c>
       <c r="D66" t="s">
-        <v>36</v>
+        <v>80</v>
       </c>
       <c r="E66" t="s">
         <v>233</v>
       </c>
-      <c r="F66" s="15" t="s">
-        <v>179</v>
-      </c>
-      <c r="G66" s="15" t="s">
-        <v>177</v>
+      <c r="F66" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="G66" s="12" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A67">
-        <v>1935968</v>
+      <c r="A67" s="13" t="s">
+        <v>50</v>
       </c>
       <c r="D67" t="s">
-        <v>80</v>
+        <v>45</v>
       </c>
       <c r="E67" t="s">
+        <v>50</v>
+      </c>
+      <c r="F67" s="12" t="s">
+        <v>176</v>
+      </c>
+      <c r="G67" s="12" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A68" s="13" t="s">
         <v>234</v>
       </c>
-      <c r="F67" s="15" t="s">
-        <v>179</v>
-      </c>
-      <c r="G67" s="15" t="s">
-        <v>180</v>
+      <c r="D68" t="s">
+        <v>7</v>
+      </c>
+      <c r="F68" s="12" t="s">
+        <v>176</v>
+      </c>
+      <c r="G68" s="12" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A69" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="D69" t="s">
+        <v>45</v>
+      </c>
+      <c r="E69" t="s">
+        <v>51</v>
+      </c>
+      <c r="F69" s="12" t="s">
+        <v>176</v>
+      </c>
+      <c r="G69" s="12" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A70" s="13" t="s">
+        <v>235</v>
+      </c>
+      <c r="D70" t="s">
+        <v>44</v>
+      </c>
+      <c r="F70" s="12" t="s">
+        <v>176</v>
+      </c>
+      <c r="G70" s="12" t="s">
+        <v>177</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G61" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:G60" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" sqref="F2:F686" xr:uid="{00000000-0002-0000-0100-000002000000}">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F685" xr:uid="{00000000-0002-0000-0100-000002000000}">
       <formula1>"Caja de Ahorro,Tarjeta de crédito"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="G2:G686" xr:uid="{00000000-0002-0000-0100-000003000000}">
+    <dataValidation type="list" allowBlank="1" sqref="G2:G685" xr:uid="{00000000-0002-0000-0100-000003000000}">
       <formula1>"Ingresos,Gastos"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2658,13 +2702,13 @@
           <x14:formula1>
             <xm:f>Categorías!$A$2:$A$27</xm:f>
           </x14:formula1>
-          <xm:sqref>D2:D686</xm:sqref>
+          <xm:sqref>D2:D685</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0100-000001000000}">
           <x14:formula1>
             <xm:f>Categorías!$D$2:$D$62</xm:f>
           </x14:formula1>
-          <xm:sqref>E2:E686</xm:sqref>
+          <xm:sqref>E2:E685</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>